<commit_message>
Add maternal coverage and update Figure 3
Add maternal immunization coverage data and generate Table S1; update Figure 3 generation. Adds Data/maternal immunization coverage.xlsx and Output/Table S1.csv, updates Output/Figure 3.{pdf,png,xlsx}, and refactors Script/figure3.R to read and clean coverage data, extract latest country-level coverage, join with mapping data, add a density inset and coverage choropleth, simplify the timing panel, adjust layout/coords, and save the combined figure and updated Excel sheets. Also updates saved figure dimensions and last edit time in the script.
</commit_message>
<xml_diff>
--- a/Output/Figure 3.xlsx
+++ b/Output/Figure 3.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="843" uniqueCount="843">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="890" uniqueCount="890">
   <si>
     <t xml:space="preserve">CODE</t>
   </si>
@@ -2543,6 +2543,147 @@
   </si>
   <si>
     <t xml:space="preserve">VaccinePregnantTime2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">YEAR</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Coverage</t>
+  </si>
+  <si>
+    <t xml:space="preserve">COVERAGE_CATEGORY_DESCRIPTION</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NAME</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2024</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Administrative coverage; Official coverage</t>
+  </si>
+  <si>
+    <t xml:space="preserve">argentina</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2023</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Article</t>
+  </si>
+  <si>
+    <t xml:space="preserve">australia</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2014-2015</t>
+  </si>
+  <si>
+    <t xml:space="preserve">belgium</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2022</t>
+  </si>
+  <si>
+    <t xml:space="preserve">bahrain</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Administrative coverage</t>
+  </si>
+  <si>
+    <t xml:space="preserve">bahamas</t>
+  </si>
+  <si>
+    <t xml:space="preserve">bermuda</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Administrative coverage; Article</t>
+  </si>
+  <si>
+    <t xml:space="preserve">brazil</t>
+  </si>
+  <si>
+    <t xml:space="preserve">canada</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2021</t>
+  </si>
+  <si>
+    <t xml:space="preserve">switzerland</t>
+  </si>
+  <si>
+    <t xml:space="preserve">chile</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Official coverage</t>
+  </si>
+  <si>
+    <t xml:space="preserve">colombia</t>
+  </si>
+  <si>
+    <t xml:space="preserve">costa rica</t>
+  </si>
+  <si>
+    <t xml:space="preserve">cuba</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2020-2021</t>
+  </si>
+  <si>
+    <t xml:space="preserve">czechia</t>
+  </si>
+  <si>
+    <t xml:space="preserve">germany</t>
+  </si>
+  <si>
+    <t xml:space="preserve">dominica</t>
+  </si>
+  <si>
+    <t xml:space="preserve">denmark</t>
+  </si>
+  <si>
+    <t xml:space="preserve">dominican republic</t>
+  </si>
+  <si>
+    <t xml:space="preserve">spain</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2025</t>
+  </si>
+  <si>
+    <t xml:space="preserve">finland</t>
+  </si>
+  <si>
+    <t xml:space="preserve">france</t>
+  </si>
+  <si>
+    <t xml:space="preserve">united kingdom of great britain and northern ireland</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Official coverage; Administrative coverage</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2018</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Netherlands (Kingdom of the)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2024.5-2025.4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2023.2-2023.4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2023.3-2023.6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2018-2019</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2023.1-2023.10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2023.2-2023.5</t>
   </si>
 </sst>
 </file>
@@ -7969,6 +8110,578 @@
         <v>568</v>
       </c>
     </row>
+    <row r="23">
+      <c r="A23" t="s">
+        <v>703</v>
+      </c>
+      <c r="B23" t="s">
+        <v>565</v>
+      </c>
+      <c r="C23" t="n">
+        <v>24</v>
+      </c>
+      <c r="D23" t="n">
+        <v>36</v>
+      </c>
+      <c r="E23" t="n">
+        <v>55</v>
+      </c>
+      <c r="F23" t="s">
+        <v>704</v>
+      </c>
+      <c r="G23" t="s">
+        <v>705</v>
+      </c>
+      <c r="H23" t="s">
+        <v>706</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="s">
+        <v>824</v>
+      </c>
+      <c r="B24" t="s">
+        <v>825</v>
+      </c>
+      <c r="C24" t="n">
+        <v>26</v>
+      </c>
+      <c r="D24" t="n">
+        <v>34</v>
+      </c>
+      <c r="E24" t="n">
+        <v>196</v>
+      </c>
+      <c r="F24" t="s">
+        <v>826</v>
+      </c>
+      <c r="G24" t="s">
+        <v>827</v>
+      </c>
+      <c r="H24" t="s">
+        <v>828</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="s">
+        <v>176</v>
+      </c>
+      <c r="B25" t="s">
+        <v>177</v>
+      </c>
+      <c r="C25" t="n">
+        <v>26</v>
+      </c>
+      <c r="D25" t="n">
+        <v>36</v>
+      </c>
+      <c r="E25" t="n">
+        <v>125</v>
+      </c>
+      <c r="F25" t="s">
+        <v>178</v>
+      </c>
+      <c r="G25" t="s">
+        <v>179</v>
+      </c>
+      <c r="H25" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="s">
+        <v>137</v>
+      </c>
+      <c r="B26" t="s">
+        <v>138</v>
+      </c>
+      <c r="C26" t="n">
+        <v>27</v>
+      </c>
+      <c r="D26" t="n">
+        <v>32</v>
+      </c>
+      <c r="E26" t="n">
+        <v>101</v>
+      </c>
+      <c r="F26" t="s">
+        <v>139</v>
+      </c>
+      <c r="G26" t="s">
+        <v>140</v>
+      </c>
+      <c r="H26" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="s">
+        <v>22</v>
+      </c>
+      <c r="B27" t="s">
+        <v>24</v>
+      </c>
+      <c r="C27" t="n">
+        <v>27</v>
+      </c>
+      <c r="D27" t="n">
+        <v>36</v>
+      </c>
+      <c r="E27" t="n">
+        <v>74</v>
+      </c>
+      <c r="F27" t="s">
+        <v>25</v>
+      </c>
+      <c r="G27" t="s">
+        <v>26</v>
+      </c>
+      <c r="H27" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="s">
+        <v>50</v>
+      </c>
+      <c r="B28" t="s">
+        <v>24</v>
+      </c>
+      <c r="C28" t="n">
+        <v>27</v>
+      </c>
+      <c r="D28" t="n">
+        <v>36</v>
+      </c>
+      <c r="E28" t="n">
+        <v>75</v>
+      </c>
+      <c r="F28" t="s">
+        <v>51</v>
+      </c>
+      <c r="G28" t="s">
+        <v>52</v>
+      </c>
+      <c r="H28" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="s">
+        <v>199</v>
+      </c>
+      <c r="B29" t="s">
+        <v>24</v>
+      </c>
+      <c r="C29" t="n">
+        <v>27</v>
+      </c>
+      <c r="D29" t="n">
+        <v>36</v>
+      </c>
+      <c r="E29" t="n">
+        <v>77</v>
+      </c>
+      <c r="F29" t="s">
+        <v>200</v>
+      </c>
+      <c r="G29" t="s">
+        <v>201</v>
+      </c>
+      <c r="H29" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="s">
+        <v>223</v>
+      </c>
+      <c r="B30" t="s">
+        <v>24</v>
+      </c>
+      <c r="C30" t="n">
+        <v>27</v>
+      </c>
+      <c r="D30" t="n">
+        <v>36</v>
+      </c>
+      <c r="E30" t="n">
+        <v>111</v>
+      </c>
+      <c r="F30" t="s">
+        <v>224</v>
+      </c>
+      <c r="G30" t="s">
+        <v>225</v>
+      </c>
+      <c r="H30" t="s">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="s">
+        <v>243</v>
+      </c>
+      <c r="B31" t="s">
+        <v>24</v>
+      </c>
+      <c r="C31" t="n">
+        <v>27</v>
+      </c>
+      <c r="D31" t="n">
+        <v>36</v>
+      </c>
+      <c r="E31" t="n">
+        <v>92</v>
+      </c>
+      <c r="F31" t="s">
+        <v>244</v>
+      </c>
+      <c r="G31" t="s">
+        <v>245</v>
+      </c>
+      <c r="H31" t="s">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="s">
+        <v>345</v>
+      </c>
+      <c r="B32" t="s">
+        <v>24</v>
+      </c>
+      <c r="C32" t="n">
+        <v>27</v>
+      </c>
+      <c r="D32" t="n">
+        <v>36</v>
+      </c>
+      <c r="E32" t="n">
+        <v>163</v>
+      </c>
+      <c r="F32" t="s">
+        <v>346</v>
+      </c>
+      <c r="G32" t="s">
+        <v>347</v>
+      </c>
+      <c r="H32" t="s">
+        <v>348</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="s">
+        <v>367</v>
+      </c>
+      <c r="B33" t="s">
+        <v>24</v>
+      </c>
+      <c r="C33" t="n">
+        <v>27</v>
+      </c>
+      <c r="D33" t="n">
+        <v>36</v>
+      </c>
+      <c r="E33" t="n">
+        <v>85</v>
+      </c>
+      <c r="F33" t="s">
+        <v>368</v>
+      </c>
+      <c r="G33" t="s">
+        <v>369</v>
+      </c>
+      <c r="H33" t="s">
+        <v>370</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="s">
+        <v>447</v>
+      </c>
+      <c r="B34" t="s">
+        <v>24</v>
+      </c>
+      <c r="C34" t="n">
+        <v>27</v>
+      </c>
+      <c r="D34" t="n">
+        <v>36</v>
+      </c>
+      <c r="E34" t="n">
+        <v>60</v>
+      </c>
+      <c r="F34" t="s">
+        <v>448</v>
+      </c>
+      <c r="G34" t="s">
+        <v>449</v>
+      </c>
+      <c r="H34" t="s">
+        <v>450</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="s">
+        <v>481</v>
+      </c>
+      <c r="B35" t="s">
+        <v>24</v>
+      </c>
+      <c r="C35" t="n">
+        <v>27</v>
+      </c>
+      <c r="D35" t="n">
+        <v>36</v>
+      </c>
+      <c r="E35" t="n">
+        <v>130</v>
+      </c>
+      <c r="F35" t="s">
+        <v>482</v>
+      </c>
+      <c r="G35" t="s">
+        <v>483</v>
+      </c>
+      <c r="H35" t="s">
+        <v>484</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="s">
+        <v>590</v>
+      </c>
+      <c r="B36" t="s">
+        <v>24</v>
+      </c>
+      <c r="C36" t="n">
+        <v>27</v>
+      </c>
+      <c r="D36" t="n">
+        <v>36</v>
+      </c>
+      <c r="E36" t="n">
+        <v>132</v>
+      </c>
+      <c r="F36" t="s">
+        <v>591</v>
+      </c>
+      <c r="G36" t="s">
+        <v>592</v>
+      </c>
+      <c r="H36" t="s">
+        <v>593</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="s">
+        <v>610</v>
+      </c>
+      <c r="B37" t="s">
+        <v>24</v>
+      </c>
+      <c r="C37" t="n">
+        <v>27</v>
+      </c>
+      <c r="D37" t="n">
+        <v>36</v>
+      </c>
+      <c r="E37" t="n">
+        <v>51</v>
+      </c>
+      <c r="F37" t="s">
+        <v>611</v>
+      </c>
+      <c r="G37" t="s">
+        <v>612</v>
+      </c>
+      <c r="H37" t="s">
+        <v>613</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="s">
+        <v>647</v>
+      </c>
+      <c r="B38" t="s">
+        <v>24</v>
+      </c>
+      <c r="C38" t="n">
+        <v>27</v>
+      </c>
+      <c r="D38" t="n">
+        <v>36</v>
+      </c>
+      <c r="E38" t="n">
+        <v>152</v>
+      </c>
+      <c r="F38" t="s">
+        <v>648</v>
+      </c>
+      <c r="G38" t="s">
+        <v>649</v>
+      </c>
+      <c r="H38" t="s">
+        <v>650</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="s">
+        <v>659</v>
+      </c>
+      <c r="B39" t="s">
+        <v>24</v>
+      </c>
+      <c r="C39" t="n">
+        <v>27</v>
+      </c>
+      <c r="D39" t="n">
+        <v>36</v>
+      </c>
+      <c r="E39" t="n">
+        <v>69</v>
+      </c>
+      <c r="F39" t="s">
+        <v>660</v>
+      </c>
+      <c r="G39" t="s">
+        <v>661</v>
+      </c>
+      <c r="H39" t="s">
+        <v>662</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="s">
+        <v>789</v>
+      </c>
+      <c r="B40" t="s">
+        <v>24</v>
+      </c>
+      <c r="C40" t="n">
+        <v>27</v>
+      </c>
+      <c r="D40" t="n">
+        <v>36</v>
+      </c>
+      <c r="E40" t="n">
+        <v>102</v>
+      </c>
+      <c r="F40" t="s">
+        <v>790</v>
+      </c>
+      <c r="G40" t="s">
+        <v>791</v>
+      </c>
+      <c r="H40" t="s">
+        <v>792</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="s">
+        <v>147</v>
+      </c>
+      <c r="B41" t="s">
+        <v>148</v>
+      </c>
+      <c r="C41" t="n">
+        <v>28</v>
+      </c>
+      <c r="D41" t="n">
+        <v>36</v>
+      </c>
+      <c r="E41" t="n">
+        <v>98</v>
+      </c>
+      <c r="F41" t="s">
+        <v>149</v>
+      </c>
+      <c r="G41" t="s">
+        <v>150</v>
+      </c>
+      <c r="H41" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="s">
+        <v>207</v>
+      </c>
+      <c r="B42" t="s">
+        <v>148</v>
+      </c>
+      <c r="C42" t="n">
+        <v>28</v>
+      </c>
+      <c r="D42" t="n">
+        <v>36</v>
+      </c>
+      <c r="E42" t="n">
+        <v>81</v>
+      </c>
+      <c r="F42" t="s">
+        <v>208</v>
+      </c>
+      <c r="G42" t="s">
+        <v>209</v>
+      </c>
+      <c r="H42" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="s">
+        <v>371</v>
+      </c>
+      <c r="B43" t="s">
+        <v>148</v>
+      </c>
+      <c r="C43" t="n">
+        <v>28</v>
+      </c>
+      <c r="D43" t="n">
+        <v>36</v>
+      </c>
+      <c r="E43" t="n">
+        <v>86</v>
+      </c>
+      <c r="F43" t="s">
+        <v>372</v>
+      </c>
+      <c r="G43" t="s">
+        <v>373</v>
+      </c>
+      <c r="H43" t="s">
+        <v>374</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="s">
+        <v>785</v>
+      </c>
+      <c r="B44" t="s">
+        <v>148</v>
+      </c>
+      <c r="C44" t="n">
+        <v>28</v>
+      </c>
+      <c r="D44" t="n">
+        <v>36</v>
+      </c>
+      <c r="E44" t="n">
+        <v>99</v>
+      </c>
+      <c r="F44" t="s">
+        <v>786</v>
+      </c>
+      <c r="G44" t="s">
+        <v>787</v>
+      </c>
+      <c r="H44" t="s">
+        <v>788</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
@@ -7985,597 +8698,1913 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>2</v>
+        <v>843</v>
       </c>
       <c r="C1" t="s">
-        <v>841</v>
+        <v>844</v>
       </c>
       <c r="D1" t="s">
-        <v>842</v>
+        <v>845</v>
       </c>
       <c r="E1" t="s">
+        <v>846</v>
+      </c>
+      <c r="F1" t="s">
         <v>3</v>
       </c>
-      <c r="F1" t="s">
+      <c r="G1" t="s">
         <v>4</v>
       </c>
-      <c r="G1" t="s">
+      <c r="H1" t="s">
         <v>5</v>
       </c>
-      <c r="H1" t="s">
+      <c r="I1" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>703</v>
+        <v>32</v>
       </c>
       <c r="B2" t="s">
-        <v>565</v>
+        <v>847</v>
       </c>
       <c r="C2" t="n">
-        <v>24</v>
-      </c>
-      <c r="D2" t="n">
+        <v>69.45</v>
+      </c>
+      <c r="D2" t="s">
+        <v>848</v>
+      </c>
+      <c r="E2" t="s">
+        <v>849</v>
+      </c>
+      <c r="F2" t="n">
+        <v>97</v>
+      </c>
+      <c r="G2" t="s">
+        <v>34</v>
+      </c>
+      <c r="H2" t="s">
+        <v>35</v>
+      </c>
+      <c r="I2" t="s">
         <v>36</v>
-      </c>
-      <c r="E2" t="n">
-        <v>55</v>
-      </c>
-      <c r="F2" t="s">
-        <v>704</v>
-      </c>
-      <c r="G2" t="s">
-        <v>705</v>
-      </c>
-      <c r="H2" t="s">
-        <v>706</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>824</v>
+        <v>45</v>
       </c>
       <c r="B3" t="s">
-        <v>825</v>
+        <v>850</v>
       </c>
       <c r="C3" t="n">
-        <v>26</v>
-      </c>
-      <c r="D3" t="n">
-        <v>34</v>
-      </c>
-      <c r="E3" t="n">
-        <v>196</v>
-      </c>
-      <c r="F3" t="s">
-        <v>826</v>
+        <v>72.9</v>
+      </c>
+      <c r="D3" t="s">
+        <v>851</v>
+      </c>
+      <c r="E3" t="s">
+        <v>852</v>
+      </c>
+      <c r="F3" t="n">
+        <v>71</v>
       </c>
       <c r="G3" t="s">
-        <v>827</v>
+        <v>47</v>
       </c>
       <c r="H3" t="s">
-        <v>828</v>
+        <v>48</v>
+      </c>
+      <c r="I3" t="s">
+        <v>49</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>176</v>
+        <v>62</v>
       </c>
       <c r="B4" t="s">
-        <v>177</v>
+        <v>853</v>
       </c>
       <c r="C4" t="n">
-        <v>26</v>
-      </c>
-      <c r="D4" t="n">
-        <v>36</v>
-      </c>
-      <c r="E4" t="n">
-        <v>125</v>
-      </c>
-      <c r="F4" t="s">
-        <v>178</v>
+        <v>64</v>
+      </c>
+      <c r="D4" t="s">
+        <v>851</v>
+      </c>
+      <c r="E4" t="s">
+        <v>854</v>
+      </c>
+      <c r="F4" t="n">
+        <v>76</v>
       </c>
       <c r="G4" t="s">
-        <v>179</v>
+        <v>64</v>
       </c>
       <c r="H4" t="s">
-        <v>180</v>
+        <v>65</v>
+      </c>
+      <c r="I4" t="s">
+        <v>66</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>137</v>
+        <v>83</v>
       </c>
       <c r="B5" t="s">
-        <v>138</v>
+        <v>855</v>
       </c>
       <c r="C5" t="n">
-        <v>27</v>
-      </c>
-      <c r="D5" t="n">
-        <v>32</v>
-      </c>
-      <c r="E5" t="n">
-        <v>101</v>
-      </c>
-      <c r="F5" t="s">
-        <v>139</v>
+        <v>13.16</v>
+      </c>
+      <c r="D5" t="s">
+        <v>848</v>
+      </c>
+      <c r="E5" t="s">
+        <v>856</v>
+      </c>
+      <c r="F5" t="n">
+        <v>140</v>
       </c>
       <c r="G5" t="s">
-        <v>140</v>
+        <v>84</v>
       </c>
       <c r="H5" t="s">
-        <v>141</v>
+        <v>85</v>
+      </c>
+      <c r="I5" t="s">
+        <v>86</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>22</v>
+        <v>87</v>
       </c>
       <c r="B6" t="s">
-        <v>24</v>
+        <v>847</v>
       </c>
       <c r="C6" t="n">
-        <v>27</v>
-      </c>
-      <c r="D6" t="n">
-        <v>36</v>
-      </c>
-      <c r="E6" t="n">
-        <v>74</v>
-      </c>
-      <c r="F6" t="s">
-        <v>25</v>
+        <v>92.34</v>
+      </c>
+      <c r="D6" t="s">
+        <v>857</v>
+      </c>
+      <c r="E6" t="s">
+        <v>858</v>
+      </c>
+      <c r="F6" t="n">
+        <v>106</v>
       </c>
       <c r="G6" t="s">
-        <v>26</v>
+        <v>89</v>
       </c>
       <c r="H6" t="s">
-        <v>27</v>
+        <v>90</v>
+      </c>
+      <c r="I6" t="s">
+        <v>91</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>50</v>
+        <v>104</v>
       </c>
       <c r="B7" t="s">
-        <v>24</v>
+        <v>855</v>
       </c>
       <c r="C7" t="n">
-        <v>27</v>
-      </c>
-      <c r="D7" t="n">
-        <v>36</v>
-      </c>
-      <c r="E7" t="n">
-        <v>75</v>
-      </c>
-      <c r="F7" t="s">
-        <v>51</v>
+        <v>18.95</v>
+      </c>
+      <c r="D7" t="s">
+        <v>857</v>
+      </c>
+      <c r="E7" t="s">
+        <v>859</v>
+      </c>
+      <c r="F7" t="n">
+        <v>305</v>
       </c>
       <c r="G7" t="s">
-        <v>52</v>
+        <v>106</v>
       </c>
       <c r="H7" t="s">
-        <v>53</v>
+        <v>107</v>
+      </c>
+      <c r="I7" t="s">
+        <v>108</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>199</v>
+        <v>113</v>
       </c>
       <c r="B8" t="s">
-        <v>24</v>
+        <v>850</v>
       </c>
       <c r="C8" t="n">
-        <v>27</v>
-      </c>
-      <c r="D8" t="n">
-        <v>36</v>
-      </c>
-      <c r="E8" t="n">
-        <v>77</v>
-      </c>
-      <c r="F8" t="s">
-        <v>200</v>
+        <v>74.005</v>
+      </c>
+      <c r="D8" t="s">
+        <v>860</v>
+      </c>
+      <c r="E8" t="s">
+        <v>861</v>
+      </c>
+      <c r="F8" t="n">
+        <v>135</v>
       </c>
       <c r="G8" t="s">
-        <v>201</v>
+        <v>114</v>
       </c>
       <c r="H8" t="s">
-        <v>202</v>
+        <v>115</v>
+      </c>
+      <c r="I8" t="s">
+        <v>116</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>223</v>
+        <v>137</v>
       </c>
       <c r="B9" t="s">
-        <v>24</v>
+        <v>847</v>
       </c>
       <c r="C9" t="n">
-        <v>27</v>
-      </c>
-      <c r="D9" t="n">
-        <v>36</v>
-      </c>
-      <c r="E9" t="n">
-        <v>111</v>
-      </c>
-      <c r="F9" t="s">
-        <v>224</v>
+        <v>65</v>
+      </c>
+      <c r="D9" t="s">
+        <v>848</v>
+      </c>
+      <c r="E9" t="s">
+        <v>862</v>
+      </c>
+      <c r="F9" t="n">
+        <v>101</v>
       </c>
       <c r="G9" t="s">
-        <v>225</v>
+        <v>139</v>
       </c>
       <c r="H9" t="s">
-        <v>226</v>
+        <v>140</v>
+      </c>
+      <c r="I9" t="s">
+        <v>141</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>243</v>
+        <v>142</v>
       </c>
       <c r="B10" t="s">
-        <v>24</v>
+        <v>863</v>
       </c>
       <c r="C10" t="n">
-        <v>27</v>
-      </c>
-      <c r="D10" t="n">
-        <v>36</v>
-      </c>
-      <c r="E10" t="n">
-        <v>92</v>
-      </c>
-      <c r="F10" t="s">
-        <v>244</v>
+        <v>85</v>
+      </c>
+      <c r="D10" t="s">
+        <v>851</v>
+      </c>
+      <c r="E10" t="s">
+        <v>864</v>
+      </c>
+      <c r="F10" t="n">
+        <v>94</v>
       </c>
       <c r="G10" t="s">
-        <v>245</v>
+        <v>144</v>
       </c>
       <c r="H10" t="s">
-        <v>246</v>
+        <v>145</v>
+      </c>
+      <c r="I10" t="s">
+        <v>146</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>345</v>
+        <v>147</v>
       </c>
       <c r="B11" t="s">
-        <v>24</v>
+        <v>847</v>
       </c>
       <c r="C11" t="n">
-        <v>27</v>
-      </c>
-      <c r="D11" t="n">
-        <v>36</v>
-      </c>
-      <c r="E11" t="n">
-        <v>163</v>
-      </c>
-      <c r="F11" t="s">
-        <v>346</v>
+        <v>65.49</v>
+      </c>
+      <c r="D11" t="s">
+        <v>857</v>
+      </c>
+      <c r="E11" t="s">
+        <v>865</v>
+      </c>
+      <c r="F11" t="n">
+        <v>98</v>
       </c>
       <c r="G11" t="s">
-        <v>347</v>
+        <v>149</v>
       </c>
       <c r="H11" t="s">
-        <v>348</v>
+        <v>150</v>
+      </c>
+      <c r="I11" t="s">
+        <v>151</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>367</v>
+        <v>176</v>
       </c>
       <c r="B12" t="s">
-        <v>24</v>
+        <v>847</v>
       </c>
       <c r="C12" t="n">
-        <v>27</v>
-      </c>
-      <c r="D12" t="n">
-        <v>36</v>
-      </c>
-      <c r="E12" t="n">
-        <v>85</v>
-      </c>
-      <c r="F12" t="s">
-        <v>368</v>
+        <v>74</v>
+      </c>
+      <c r="D12" t="s">
+        <v>866</v>
+      </c>
+      <c r="E12" t="s">
+        <v>867</v>
+      </c>
+      <c r="F12" t="n">
+        <v>125</v>
       </c>
       <c r="G12" t="s">
-        <v>369</v>
+        <v>178</v>
       </c>
       <c r="H12" t="s">
-        <v>370</v>
+        <v>179</v>
+      </c>
+      <c r="I12" t="s">
+        <v>180</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>447</v>
+        <v>189</v>
       </c>
       <c r="B13" t="s">
-        <v>24</v>
+        <v>847</v>
       </c>
       <c r="C13" t="n">
-        <v>27</v>
-      </c>
-      <c r="D13" t="n">
-        <v>36</v>
-      </c>
-      <c r="E13" t="n">
-        <v>60</v>
-      </c>
-      <c r="F13" t="s">
-        <v>448</v>
+        <v>95.42</v>
+      </c>
+      <c r="D13" t="s">
+        <v>857</v>
+      </c>
+      <c r="E13" t="s">
+        <v>868</v>
+      </c>
+      <c r="F13" t="n">
+        <v>126</v>
       </c>
       <c r="G13" t="s">
-        <v>449</v>
+        <v>190</v>
       </c>
       <c r="H13" t="s">
-        <v>450</v>
+        <v>191</v>
+      </c>
+      <c r="I13" t="s">
+        <v>192</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>481</v>
+        <v>193</v>
       </c>
       <c r="B14" t="s">
-        <v>24</v>
+        <v>863</v>
       </c>
       <c r="C14" t="n">
-        <v>27</v>
-      </c>
-      <c r="D14" t="n">
-        <v>36</v>
-      </c>
-      <c r="E14" t="n">
-        <v>130</v>
-      </c>
-      <c r="F14" t="s">
-        <v>482</v>
+        <v>100</v>
+      </c>
+      <c r="D14" t="s">
+        <v>848</v>
+      </c>
+      <c r="E14" t="s">
+        <v>869</v>
+      </c>
+      <c r="F14" t="n">
+        <v>109</v>
       </c>
       <c r="G14" t="s">
-        <v>483</v>
+        <v>194</v>
       </c>
       <c r="H14" t="s">
-        <v>484</v>
+        <v>195</v>
+      </c>
+      <c r="I14" t="s">
+        <v>196</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>590</v>
+        <v>203</v>
       </c>
       <c r="B15" t="s">
-        <v>24</v>
+        <v>870</v>
       </c>
       <c r="C15" t="n">
-        <v>27</v>
-      </c>
-      <c r="D15" t="n">
-        <v>36</v>
-      </c>
-      <c r="E15" t="n">
-        <v>132</v>
-      </c>
-      <c r="F15" t="s">
-        <v>591</v>
+        <v>1.6</v>
+      </c>
+      <c r="D15" t="s">
+        <v>851</v>
+      </c>
+      <c r="E15" t="s">
+        <v>871</v>
+      </c>
+      <c r="F15" t="n">
+        <v>47</v>
       </c>
       <c r="G15" t="s">
-        <v>592</v>
+        <v>204</v>
       </c>
       <c r="H15" t="s">
-        <v>593</v>
+        <v>205</v>
+      </c>
+      <c r="I15" t="s">
+        <v>206</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>610</v>
+        <v>207</v>
       </c>
       <c r="B16" t="s">
-        <v>24</v>
+        <v>847</v>
       </c>
       <c r="C16" t="n">
-        <v>27</v>
-      </c>
-      <c r="D16" t="n">
-        <v>36</v>
-      </c>
-      <c r="E16" t="n">
-        <v>51</v>
-      </c>
-      <c r="F16" t="s">
-        <v>611</v>
+        <v>47.9</v>
+      </c>
+      <c r="D16" t="s">
+        <v>848</v>
+      </c>
+      <c r="E16" t="s">
+        <v>872</v>
+      </c>
+      <c r="F16" t="n">
+        <v>81</v>
       </c>
       <c r="G16" t="s">
-        <v>612</v>
+        <v>208</v>
       </c>
       <c r="H16" t="s">
-        <v>613</v>
+        <v>209</v>
+      </c>
+      <c r="I16" t="s">
+        <v>210</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>647</v>
+        <v>215</v>
       </c>
       <c r="B17" t="s">
-        <v>24</v>
+        <v>847</v>
       </c>
       <c r="C17" t="n">
-        <v>27</v>
-      </c>
-      <c r="D17" t="n">
-        <v>36</v>
-      </c>
-      <c r="E17" t="n">
-        <v>152</v>
-      </c>
-      <c r="F17" t="s">
-        <v>648</v>
+        <v>48.17</v>
+      </c>
+      <c r="D17" t="s">
+        <v>866</v>
+      </c>
+      <c r="E17" t="s">
+        <v>873</v>
+      </c>
+      <c r="F17" t="n">
+        <v>110</v>
       </c>
       <c r="G17" t="s">
-        <v>649</v>
+        <v>216</v>
       </c>
       <c r="H17" t="s">
-        <v>650</v>
+        <v>217</v>
+      </c>
+      <c r="I17" t="s">
+        <v>218</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>659</v>
+        <v>219</v>
       </c>
       <c r="B18" t="s">
-        <v>24</v>
+        <v>847</v>
       </c>
       <c r="C18" t="n">
-        <v>27</v>
-      </c>
-      <c r="D18" t="n">
-        <v>36</v>
-      </c>
-      <c r="E18" t="n">
-        <v>69</v>
-      </c>
-      <c r="F18" t="s">
-        <v>660</v>
+        <v>52.03</v>
+      </c>
+      <c r="D18" t="s">
+        <v>848</v>
+      </c>
+      <c r="E18" t="s">
+        <v>874</v>
+      </c>
+      <c r="F18" t="n">
+        <v>78</v>
       </c>
       <c r="G18" t="s">
-        <v>661</v>
+        <v>220</v>
       </c>
       <c r="H18" t="s">
-        <v>662</v>
+        <v>221</v>
+      </c>
+      <c r="I18" t="s">
+        <v>222</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>789</v>
+        <v>223</v>
       </c>
       <c r="B19" t="s">
-        <v>24</v>
+        <v>847</v>
       </c>
       <c r="C19" t="n">
-        <v>27</v>
-      </c>
-      <c r="D19" t="n">
-        <v>36</v>
-      </c>
-      <c r="E19" t="n">
-        <v>102</v>
-      </c>
-      <c r="F19" t="s">
-        <v>790</v>
+        <v>53.31</v>
+      </c>
+      <c r="D19" t="s">
+        <v>857</v>
+      </c>
+      <c r="E19" t="s">
+        <v>875</v>
+      </c>
+      <c r="F19" t="n">
+        <v>111</v>
       </c>
       <c r="G19" t="s">
-        <v>791</v>
+        <v>224</v>
       </c>
       <c r="H19" t="s">
-        <v>792</v>
+        <v>225</v>
+      </c>
+      <c r="I19" t="s">
+        <v>226</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>147</v>
+        <v>243</v>
       </c>
       <c r="B20" t="s">
-        <v>148</v>
+        <v>847</v>
       </c>
       <c r="C20" t="n">
-        <v>28</v>
-      </c>
-      <c r="D20" t="n">
-        <v>36</v>
-      </c>
-      <c r="E20" t="n">
-        <v>98</v>
-      </c>
-      <c r="F20" t="s">
-        <v>149</v>
+        <v>91.83</v>
+      </c>
+      <c r="D20" t="s">
+        <v>848</v>
+      </c>
+      <c r="E20" t="s">
+        <v>876</v>
+      </c>
+      <c r="F20" t="n">
+        <v>92</v>
       </c>
       <c r="G20" t="s">
-        <v>150</v>
+        <v>244</v>
       </c>
       <c r="H20" t="s">
-        <v>151</v>
+        <v>245</v>
+      </c>
+      <c r="I20" t="s">
+        <v>246</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="s">
-        <v>207</v>
+        <v>255</v>
       </c>
       <c r="B21" t="s">
-        <v>148</v>
+        <v>877</v>
       </c>
       <c r="C21" t="n">
-        <v>28</v>
-      </c>
-      <c r="D21" t="n">
-        <v>36</v>
-      </c>
-      <c r="E21" t="n">
-        <v>81</v>
-      </c>
-      <c r="F21" t="s">
-        <v>208</v>
+        <v>57</v>
+      </c>
+      <c r="D21" t="s">
+        <v>851</v>
+      </c>
+      <c r="E21" t="s">
+        <v>878</v>
+      </c>
+      <c r="F21" t="n">
+        <v>79</v>
       </c>
       <c r="G21" t="s">
-        <v>209</v>
+        <v>256</v>
       </c>
       <c r="H21" t="s">
-        <v>210</v>
+        <v>257</v>
+      </c>
+      <c r="I21" t="s">
+        <v>258</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="s">
-        <v>371</v>
+        <v>263</v>
       </c>
       <c r="B22" t="s">
-        <v>148</v>
+        <v>847</v>
       </c>
       <c r="C22" t="n">
-        <v>28</v>
-      </c>
-      <c r="D22" t="n">
-        <v>36</v>
-      </c>
-      <c r="E22" t="n">
-        <v>86</v>
-      </c>
-      <c r="F22" t="s">
-        <v>372</v>
+        <v>62.3</v>
+      </c>
+      <c r="D22" t="s">
+        <v>857</v>
+      </c>
+      <c r="E22" t="s">
+        <v>879</v>
+      </c>
+      <c r="F22" t="n">
+        <v>80</v>
       </c>
       <c r="G22" t="s">
-        <v>373</v>
+        <v>264</v>
       </c>
       <c r="H22" t="s">
-        <v>374</v>
+        <v>265</v>
+      </c>
+      <c r="I22" t="s">
+        <v>266</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="s">
+        <v>275</v>
+      </c>
+      <c r="B23" t="s">
+        <v>847</v>
+      </c>
+      <c r="C23" t="n">
+        <v>58.56</v>
+      </c>
+      <c r="D23" t="s">
+        <v>848</v>
+      </c>
+      <c r="E23" t="s">
+        <v>880</v>
+      </c>
+      <c r="F23" t="n">
+        <v>95</v>
+      </c>
+      <c r="G23" t="s">
+        <v>277</v>
+      </c>
+      <c r="H23" t="s">
+        <v>278</v>
+      </c>
+      <c r="I23" t="s">
+        <v>279</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="s">
+        <v>292</v>
+      </c>
+      <c r="B24" t="s">
+        <v>863</v>
+      </c>
+      <c r="C24" t="n">
+        <v>54.23</v>
+      </c>
+      <c r="D24" t="s">
+        <v>857</v>
+      </c>
+      <c r="E24" t="s">
+        <v>294</v>
+      </c>
+      <c r="F24" t="n">
+        <v>206</v>
+      </c>
+      <c r="G24" t="s">
+        <v>293</v>
+      </c>
+      <c r="H24" t="s">
+        <v>294</v>
+      </c>
+      <c r="I24" t="s">
+        <v>295</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="s">
+        <v>296</v>
+      </c>
+      <c r="B25" t="s">
+        <v>850</v>
+      </c>
+      <c r="C25" t="n">
+        <v>86.92</v>
+      </c>
+      <c r="D25" t="s">
+        <v>857</v>
+      </c>
+      <c r="E25" t="s">
+        <v>298</v>
+      </c>
+      <c r="F25" t="n">
+        <v>209</v>
+      </c>
+      <c r="G25" t="s">
+        <v>297</v>
+      </c>
+      <c r="H25" t="s">
+        <v>298</v>
+      </c>
+      <c r="I25" t="s">
+        <v>299</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="s">
+        <v>304</v>
+      </c>
+      <c r="B26" t="s">
+        <v>877</v>
+      </c>
+      <c r="C26" t="n">
+        <v>16.8</v>
+      </c>
+      <c r="D26" t="s">
+        <v>851</v>
+      </c>
+      <c r="E26" t="s">
+        <v>306</v>
+      </c>
+      <c r="F26" t="n">
+        <v>82</v>
+      </c>
+      <c r="G26" t="s">
+        <v>305</v>
+      </c>
+      <c r="H26" t="s">
+        <v>306</v>
+      </c>
+      <c r="I26" t="s">
+        <v>307</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="s">
+        <v>312</v>
+      </c>
+      <c r="B27" t="s">
+        <v>847</v>
+      </c>
+      <c r="C27" t="n">
+        <v>54.56</v>
+      </c>
+      <c r="D27" t="s">
+        <v>857</v>
+      </c>
+      <c r="E27" t="s">
+        <v>314</v>
+      </c>
+      <c r="F27" t="n">
+        <v>128</v>
+      </c>
+      <c r="G27" t="s">
+        <v>313</v>
+      </c>
+      <c r="H27" t="s">
+        <v>314</v>
+      </c>
+      <c r="I27" t="s">
+        <v>315</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="s">
+        <v>316</v>
+      </c>
+      <c r="B28" t="s">
+        <v>847</v>
+      </c>
+      <c r="C28" t="n">
+        <v>59.6</v>
+      </c>
+      <c r="D28" t="s">
+        <v>866</v>
+      </c>
+      <c r="E28" t="s">
+        <v>318</v>
+      </c>
+      <c r="F28" t="n">
+        <v>351</v>
+      </c>
+      <c r="G28" t="s">
+        <v>317</v>
+      </c>
+      <c r="H28" t="s">
+        <v>318</v>
+      </c>
+      <c r="I28" t="s">
+        <v>319</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="s">
+        <v>325</v>
+      </c>
+      <c r="B29" t="s">
+        <v>847</v>
+      </c>
+      <c r="C29" t="n">
+        <v>79.405</v>
+      </c>
+      <c r="D29" t="s">
+        <v>881</v>
+      </c>
+      <c r="E29" t="s">
+        <v>327</v>
+      </c>
+      <c r="F29" t="n">
+        <v>129</v>
+      </c>
+      <c r="G29" t="s">
+        <v>326</v>
+      </c>
+      <c r="H29" t="s">
+        <v>327</v>
+      </c>
+      <c r="I29" t="s">
+        <v>328</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="s">
+        <v>333</v>
+      </c>
+      <c r="B30" t="s">
+        <v>847</v>
+      </c>
+      <c r="C30" t="n">
+        <v>39.07</v>
+      </c>
+      <c r="D30" t="s">
+        <v>866</v>
+      </c>
+      <c r="E30" t="s">
+        <v>335</v>
+      </c>
+      <c r="F30" t="n">
+        <v>114</v>
+      </c>
+      <c r="G30" t="s">
+        <v>334</v>
+      </c>
+      <c r="H30" t="s">
+        <v>335</v>
+      </c>
+      <c r="I30" t="s">
+        <v>336</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="s">
+        <v>349</v>
+      </c>
+      <c r="B31" t="s">
+        <v>882</v>
+      </c>
+      <c r="C31" t="n">
+        <v>49</v>
+      </c>
+      <c r="D31" t="s">
+        <v>851</v>
+      </c>
+      <c r="E31" t="s">
+        <v>352</v>
+      </c>
+      <c r="F31" t="n">
+        <v>84</v>
+      </c>
+      <c r="G31" t="s">
+        <v>351</v>
+      </c>
+      <c r="H31" t="s">
+        <v>352</v>
+      </c>
+      <c r="I31" t="s">
+        <v>353</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="s">
+        <v>367</v>
+      </c>
+      <c r="B32" t="s">
+        <v>863</v>
+      </c>
+      <c r="C32" t="n">
+        <v>49</v>
+      </c>
+      <c r="D32" t="s">
+        <v>851</v>
+      </c>
+      <c r="E32" t="s">
+        <v>369</v>
+      </c>
+      <c r="F32" t="n">
+        <v>85</v>
+      </c>
+      <c r="G32" t="s">
+        <v>368</v>
+      </c>
+      <c r="H32" t="s">
+        <v>369</v>
+      </c>
+      <c r="I32" t="s">
+        <v>370</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="s">
+        <v>371</v>
+      </c>
+      <c r="B33" t="s">
+        <v>850</v>
+      </c>
+      <c r="C33" t="n">
+        <v>79.52</v>
+      </c>
+      <c r="D33" t="s">
+        <v>851</v>
+      </c>
+      <c r="E33" t="s">
+        <v>373</v>
+      </c>
+      <c r="F33" t="n">
+        <v>86</v>
+      </c>
+      <c r="G33" t="s">
+        <v>372</v>
+      </c>
+      <c r="H33" t="s">
+        <v>373</v>
+      </c>
+      <c r="I33" t="s">
+        <v>374</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="s">
+        <v>481</v>
+      </c>
+      <c r="B34" t="s">
+        <v>850</v>
+      </c>
+      <c r="C34" t="n">
+        <v>52.44</v>
+      </c>
+      <c r="D34" t="s">
+        <v>851</v>
+      </c>
+      <c r="E34" t="s">
+        <v>483</v>
+      </c>
+      <c r="F34" t="n">
+        <v>130</v>
+      </c>
+      <c r="G34" t="s">
+        <v>482</v>
+      </c>
+      <c r="H34" t="s">
+        <v>483</v>
+      </c>
+      <c r="I34" t="s">
+        <v>484</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="s">
+        <v>493</v>
+      </c>
+      <c r="B35" t="s">
+        <v>847</v>
+      </c>
+      <c r="C35" t="n">
+        <v>29.1</v>
+      </c>
+      <c r="D35" t="s">
+        <v>857</v>
+      </c>
+      <c r="E35" t="s">
+        <v>495</v>
+      </c>
+      <c r="F35" t="n">
+        <v>211</v>
+      </c>
+      <c r="G35" t="s">
+        <v>494</v>
+      </c>
+      <c r="H35" t="s">
+        <v>495</v>
+      </c>
+      <c r="I35" t="s">
+        <v>496</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="s">
+        <v>513</v>
+      </c>
+      <c r="B36" t="s">
+        <v>847</v>
+      </c>
+      <c r="C36" t="n">
+        <v>59.6</v>
+      </c>
+      <c r="D36" t="s">
+        <v>866</v>
+      </c>
+      <c r="E36" t="s">
+        <v>515</v>
+      </c>
+      <c r="F36" t="n">
+        <v>376</v>
+      </c>
+      <c r="G36" t="s">
+        <v>514</v>
+      </c>
+      <c r="H36" t="s">
+        <v>515</v>
+      </c>
+      <c r="I36" t="s">
+        <v>516</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="s">
+        <v>526</v>
+      </c>
+      <c r="B37" t="s">
+        <v>847</v>
+      </c>
+      <c r="C37" t="n">
+        <v>60.58</v>
+      </c>
+      <c r="D37" t="s">
+        <v>857</v>
+      </c>
+      <c r="E37" t="s">
+        <v>528</v>
+      </c>
+      <c r="F37" t="n">
+        <v>183</v>
+      </c>
+      <c r="G37" t="s">
+        <v>527</v>
+      </c>
+      <c r="H37" t="s">
+        <v>528</v>
+      </c>
+      <c r="I37" t="s">
+        <v>529</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="s">
+        <v>551</v>
+      </c>
+      <c r="B38" t="s">
+        <v>850</v>
+      </c>
+      <c r="C38" t="n">
+        <v>40.98</v>
+      </c>
+      <c r="D38" t="s">
+        <v>857</v>
+      </c>
+      <c r="E38" t="s">
+        <v>553</v>
+      </c>
+      <c r="F38" t="n">
+        <v>131</v>
+      </c>
+      <c r="G38" t="s">
+        <v>552</v>
+      </c>
+      <c r="H38" t="s">
+        <v>553</v>
+      </c>
+      <c r="I38" t="s">
+        <v>554</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="s">
+        <v>559</v>
+      </c>
+      <c r="B39" t="s">
+        <v>847</v>
+      </c>
+      <c r="C39" t="n">
+        <v>66.84</v>
+      </c>
+      <c r="D39" t="s">
+        <v>881</v>
+      </c>
+      <c r="E39" t="s">
+        <v>883</v>
+      </c>
+      <c r="F39" t="n">
+        <v>89</v>
+      </c>
+      <c r="G39" t="s">
+        <v>561</v>
+      </c>
+      <c r="H39" t="s">
+        <v>562</v>
+      </c>
+      <c r="I39" t="s">
+        <v>563</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="s">
+        <v>564</v>
+      </c>
+      <c r="B40" t="s">
+        <v>884</v>
+      </c>
+      <c r="C40" t="n">
+        <v>73</v>
+      </c>
+      <c r="D40" t="s">
+        <v>851</v>
+      </c>
+      <c r="E40" t="s">
+        <v>567</v>
+      </c>
+      <c r="F40" t="n">
+        <v>90</v>
+      </c>
+      <c r="G40" t="s">
+        <v>566</v>
+      </c>
+      <c r="H40" t="s">
+        <v>567</v>
+      </c>
+      <c r="I40" t="s">
+        <v>568</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="s">
+        <v>577</v>
+      </c>
+      <c r="B41" t="s">
+        <v>850</v>
+      </c>
+      <c r="C41" t="n">
+        <v>61.25</v>
+      </c>
+      <c r="D41" t="s">
+        <v>851</v>
+      </c>
+      <c r="E41" t="s">
+        <v>580</v>
+      </c>
+      <c r="F41" t="n">
+        <v>72</v>
+      </c>
+      <c r="G41" t="s">
+        <v>579</v>
+      </c>
+      <c r="H41" t="s">
+        <v>580</v>
+      </c>
+      <c r="I41" t="s">
+        <v>581</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="s">
+        <v>582</v>
+      </c>
+      <c r="B42" t="s">
+        <v>847</v>
+      </c>
+      <c r="C42" t="n">
+        <v>92.98</v>
+      </c>
+      <c r="D42" t="s">
+        <v>848</v>
+      </c>
+      <c r="E42" t="s">
+        <v>584</v>
+      </c>
+      <c r="F42" t="n">
+        <v>150</v>
+      </c>
+      <c r="G42" t="s">
+        <v>583</v>
+      </c>
+      <c r="H42" t="s">
+        <v>584</v>
+      </c>
+      <c r="I42" t="s">
+        <v>585</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="s">
+        <v>590</v>
+      </c>
+      <c r="B43" t="s">
+        <v>847</v>
+      </c>
+      <c r="C43" t="n">
+        <v>74.29</v>
+      </c>
+      <c r="D43" t="s">
+        <v>848</v>
+      </c>
+      <c r="E43" t="s">
+        <v>592</v>
+      </c>
+      <c r="F43" t="n">
+        <v>132</v>
+      </c>
+      <c r="G43" t="s">
+        <v>591</v>
+      </c>
+      <c r="H43" t="s">
+        <v>592</v>
+      </c>
+      <c r="I43" t="s">
+        <v>593</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="s">
+        <v>594</v>
+      </c>
+      <c r="B44" t="s">
+        <v>847</v>
+      </c>
+      <c r="C44" t="n">
+        <v>93.21</v>
+      </c>
+      <c r="D44" t="s">
+        <v>857</v>
+      </c>
+      <c r="E44" t="s">
+        <v>596</v>
+      </c>
+      <c r="F44" t="n">
+        <v>123</v>
+      </c>
+      <c r="G44" t="s">
+        <v>595</v>
+      </c>
+      <c r="H44" t="s">
+        <v>596</v>
+      </c>
+      <c r="I44" t="s">
+        <v>597</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="s">
+        <v>598</v>
+      </c>
+      <c r="B45" t="s">
+        <v>855</v>
+      </c>
+      <c r="C45" t="n">
+        <v>37.41</v>
+      </c>
+      <c r="D45" t="s">
+        <v>857</v>
+      </c>
+      <c r="E45" t="s">
+        <v>600</v>
+      </c>
+      <c r="F45" t="n">
+        <v>16</v>
+      </c>
+      <c r="G45" t="s">
+        <v>599</v>
+      </c>
+      <c r="H45" t="s">
+        <v>600</v>
+      </c>
+      <c r="I45" t="s">
+        <v>601</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="s">
+        <v>610</v>
+      </c>
+      <c r="B46" t="s">
+        <v>885</v>
+      </c>
+      <c r="C46" t="n">
+        <v>23.4</v>
+      </c>
+      <c r="D46" t="s">
+        <v>851</v>
+      </c>
+      <c r="E46" t="s">
+        <v>612</v>
+      </c>
+      <c r="F46" t="n">
+        <v>51</v>
+      </c>
+      <c r="G46" t="s">
+        <v>611</v>
+      </c>
+      <c r="H46" t="s">
+        <v>612</v>
+      </c>
+      <c r="I46" t="s">
+        <v>613</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="s">
+        <v>618</v>
+      </c>
+      <c r="B47" t="s">
+        <v>847</v>
+      </c>
+      <c r="C47" t="n">
+        <v>80.4</v>
+      </c>
+      <c r="D47" t="s">
+        <v>848</v>
+      </c>
+      <c r="E47" t="s">
+        <v>620</v>
+      </c>
+      <c r="F47" t="n">
+        <v>91</v>
+      </c>
+      <c r="G47" t="s">
+        <v>619</v>
+      </c>
+      <c r="H47" t="s">
+        <v>620</v>
+      </c>
+      <c r="I47" t="s">
+        <v>621</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="s">
+        <v>622</v>
+      </c>
+      <c r="B48" t="s">
+        <v>847</v>
+      </c>
+      <c r="C48" t="n">
+        <v>62</v>
+      </c>
+      <c r="D48" t="s">
+        <v>866</v>
+      </c>
+      <c r="E48" t="s">
+        <v>624</v>
+      </c>
+      <c r="F48" t="n">
+        <v>136</v>
+      </c>
+      <c r="G48" t="s">
+        <v>623</v>
+      </c>
+      <c r="H48" t="s">
+        <v>624</v>
+      </c>
+      <c r="I48" t="s">
+        <v>625</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="s">
+        <v>647</v>
+      </c>
+      <c r="B49" t="s">
+        <v>886</v>
+      </c>
+      <c r="C49" t="n">
+        <v>3.7</v>
+      </c>
+      <c r="D49" t="s">
+        <v>851</v>
+      </c>
+      <c r="E49" t="s">
+        <v>649</v>
+      </c>
+      <c r="F49" t="n">
+        <v>152</v>
+      </c>
+      <c r="G49" t="s">
+        <v>648</v>
+      </c>
+      <c r="H49" t="s">
+        <v>649</v>
+      </c>
+      <c r="I49" t="s">
+        <v>650</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="s">
+        <v>651</v>
+      </c>
+      <c r="B50" t="s">
+        <v>855</v>
+      </c>
+      <c r="C50" t="n">
+        <v>44.05</v>
+      </c>
+      <c r="D50" t="s">
+        <v>848</v>
+      </c>
+      <c r="E50" t="s">
+        <v>653</v>
+      </c>
+      <c r="F50" t="n">
+        <v>522</v>
+      </c>
+      <c r="G50" t="s">
+        <v>652</v>
+      </c>
+      <c r="H50" t="s">
+        <v>653</v>
+      </c>
+      <c r="I50" t="s">
+        <v>654</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="s">
+        <v>659</v>
+      </c>
+      <c r="B51" t="s">
+        <v>887</v>
+      </c>
+      <c r="C51" t="n">
+        <v>25.9</v>
+      </c>
+      <c r="D51" t="s">
+        <v>851</v>
+      </c>
+      <c r="E51" t="s">
+        <v>661</v>
+      </c>
+      <c r="F51" t="n">
+        <v>69</v>
+      </c>
+      <c r="G51" t="s">
+        <v>660</v>
+      </c>
+      <c r="H51" t="s">
+        <v>661</v>
+      </c>
+      <c r="I51" t="s">
+        <v>662</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="s">
+        <v>671</v>
+      </c>
+      <c r="B52" t="s">
+        <v>847</v>
+      </c>
+      <c r="C52" t="n">
+        <v>86.48</v>
+      </c>
+      <c r="D52" t="s">
+        <v>857</v>
+      </c>
+      <c r="E52" t="s">
+        <v>673</v>
+      </c>
+      <c r="F52" t="n">
+        <v>127</v>
+      </c>
+      <c r="G52" t="s">
+        <v>672</v>
+      </c>
+      <c r="H52" t="s">
+        <v>673</v>
+      </c>
+      <c r="I52" t="s">
+        <v>674</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="s">
+        <v>699</v>
+      </c>
+      <c r="B53" t="s">
+        <v>850</v>
+      </c>
+      <c r="C53" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="D53" t="s">
+        <v>851</v>
+      </c>
+      <c r="E53" t="s">
+        <v>701</v>
+      </c>
+      <c r="F53" t="n">
+        <v>54</v>
+      </c>
+      <c r="G53" t="s">
+        <v>700</v>
+      </c>
+      <c r="H53" t="s">
+        <v>701</v>
+      </c>
+      <c r="I53" t="s">
+        <v>702</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="s">
+        <v>703</v>
+      </c>
+      <c r="B54" t="s">
+        <v>850</v>
+      </c>
+      <c r="C54" t="n">
+        <v>6.5</v>
+      </c>
+      <c r="D54" t="s">
+        <v>851</v>
+      </c>
+      <c r="E54" t="s">
+        <v>705</v>
+      </c>
+      <c r="F54" t="n">
+        <v>55</v>
+      </c>
+      <c r="G54" t="s">
+        <v>704</v>
+      </c>
+      <c r="H54" t="s">
+        <v>705</v>
+      </c>
+      <c r="I54" t="s">
+        <v>706</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="s">
+        <v>707</v>
+      </c>
+      <c r="B55" t="s">
+        <v>847</v>
+      </c>
+      <c r="C55" t="n">
+        <v>60</v>
+      </c>
+      <c r="D55" t="s">
+        <v>851</v>
+      </c>
+      <c r="E55" t="s">
+        <v>709</v>
+      </c>
+      <c r="F55" t="n">
+        <v>93</v>
+      </c>
+      <c r="G55" t="s">
+        <v>708</v>
+      </c>
+      <c r="H55" t="s">
+        <v>709</v>
+      </c>
+      <c r="I55" t="s">
+        <v>710</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="s">
+        <v>716</v>
+      </c>
+      <c r="B56" t="s">
+        <v>847</v>
+      </c>
+      <c r="C56" t="n">
+        <v>0</v>
+      </c>
+      <c r="D56" t="s">
+        <v>866</v>
+      </c>
+      <c r="E56" t="s">
+        <v>718</v>
+      </c>
+      <c r="F56" t="n">
+        <v>186</v>
+      </c>
+      <c r="G56" t="s">
+        <v>717</v>
+      </c>
+      <c r="H56" t="s">
+        <v>718</v>
+      </c>
+      <c r="I56" t="s">
+        <v>719</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="s">
+        <v>729</v>
+      </c>
+      <c r="B57" t="s">
+        <v>863</v>
+      </c>
+      <c r="C57" t="n">
+        <v>71.77</v>
+      </c>
+      <c r="D57" t="s">
+        <v>848</v>
+      </c>
+      <c r="E57" t="s">
+        <v>731</v>
+      </c>
+      <c r="F57" t="n">
+        <v>218</v>
+      </c>
+      <c r="G57" t="s">
+        <v>730</v>
+      </c>
+      <c r="H57" t="s">
+        <v>731</v>
+      </c>
+      <c r="I57" t="s">
+        <v>732</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="s">
+        <v>733</v>
+      </c>
+      <c r="B58" t="s">
+        <v>850</v>
+      </c>
+      <c r="C58" t="n">
+        <v>0</v>
+      </c>
+      <c r="D58" t="s">
+        <v>857</v>
+      </c>
+      <c r="E58" t="s">
+        <v>735</v>
+      </c>
+      <c r="F58" t="n">
+        <v>18</v>
+      </c>
+      <c r="G58" t="s">
+        <v>734</v>
+      </c>
+      <c r="H58" t="s">
+        <v>735</v>
+      </c>
+      <c r="I58" t="s">
+        <v>736</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="s">
+        <v>757</v>
+      </c>
+      <c r="B59" t="s">
+        <v>847</v>
+      </c>
+      <c r="C59" t="n">
+        <v>17.14</v>
+      </c>
+      <c r="D59" t="s">
+        <v>857</v>
+      </c>
+      <c r="E59" t="s">
+        <v>759</v>
+      </c>
+      <c r="F59" t="n">
+        <v>119</v>
+      </c>
+      <c r="G59" t="s">
+        <v>758</v>
+      </c>
+      <c r="H59" t="s">
+        <v>759</v>
+      </c>
+      <c r="I59" t="s">
+        <v>760</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="s">
+        <v>765</v>
+      </c>
+      <c r="B60" t="s">
+        <v>888</v>
+      </c>
+      <c r="C60" t="n">
+        <v>11.7</v>
+      </c>
+      <c r="D60" t="s">
+        <v>851</v>
+      </c>
+      <c r="E60" t="s">
+        <v>767</v>
+      </c>
+      <c r="F60" t="n">
+        <v>155</v>
+      </c>
+      <c r="G60" t="s">
+        <v>766</v>
+      </c>
+      <c r="H60" t="s">
+        <v>767</v>
+      </c>
+      <c r="I60" t="s">
+        <v>768</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="s">
+        <v>777</v>
+      </c>
+      <c r="B61" t="s">
+        <v>850</v>
+      </c>
+      <c r="C61" t="n">
+        <v>83</v>
+      </c>
+      <c r="D61" t="s">
+        <v>866</v>
+      </c>
+      <c r="E61" t="s">
+        <v>779</v>
+      </c>
+      <c r="F61" t="n">
+        <v>190</v>
+      </c>
+      <c r="G61" t="s">
+        <v>778</v>
+      </c>
+      <c r="H61" t="s">
+        <v>779</v>
+      </c>
+      <c r="I61" t="s">
+        <v>780</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="s">
         <v>785</v>
       </c>
-      <c r="B23" t="s">
-        <v>148</v>
-      </c>
-      <c r="C23" t="n">
-        <v>28</v>
-      </c>
-      <c r="D23" t="n">
-        <v>36</v>
-      </c>
-      <c r="E23" t="n">
+      <c r="B62" t="s">
+        <v>847</v>
+      </c>
+      <c r="C62" t="n">
+        <v>83.89</v>
+      </c>
+      <c r="D62" t="s">
+        <v>857</v>
+      </c>
+      <c r="E62" t="s">
+        <v>787</v>
+      </c>
+      <c r="F62" t="n">
         <v>99</v>
       </c>
-      <c r="F23" t="s">
+      <c r="G62" t="s">
         <v>786</v>
       </c>
-      <c r="G23" t="s">
+      <c r="H62" t="s">
         <v>787</v>
       </c>
-      <c r="H23" t="s">
+      <c r="I62" t="s">
         <v>788</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="s">
+        <v>789</v>
+      </c>
+      <c r="B63" t="s">
+        <v>850</v>
+      </c>
+      <c r="C63" t="n">
+        <v>57</v>
+      </c>
+      <c r="D63" t="s">
+        <v>851</v>
+      </c>
+      <c r="E63" t="s">
+        <v>791</v>
+      </c>
+      <c r="F63" t="n">
+        <v>102</v>
+      </c>
+      <c r="G63" t="s">
+        <v>790</v>
+      </c>
+      <c r="H63" t="s">
+        <v>791</v>
+      </c>
+      <c r="I63" t="s">
+        <v>792</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="s">
+        <v>793</v>
+      </c>
+      <c r="B64" t="s">
+        <v>850</v>
+      </c>
+      <c r="C64" t="n">
+        <v>0</v>
+      </c>
+      <c r="D64" t="s">
+        <v>866</v>
+      </c>
+      <c r="E64" t="s">
+        <v>795</v>
+      </c>
+      <c r="F64" t="n">
+        <v>41</v>
+      </c>
+      <c r="G64" t="s">
+        <v>794</v>
+      </c>
+      <c r="H64" t="s">
+        <v>795</v>
+      </c>
+      <c r="I64" t="s">
+        <v>796</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="s">
+        <v>806</v>
+      </c>
+      <c r="B65" t="s">
+        <v>889</v>
+      </c>
+      <c r="C65" t="n">
+        <v>54.5</v>
+      </c>
+      <c r="D65" t="s">
+        <v>851</v>
+      </c>
+      <c r="E65" t="s">
+        <v>808</v>
+      </c>
+      <c r="F65" t="n">
+        <v>20</v>
+      </c>
+      <c r="G65" t="s">
+        <v>807</v>
+      </c>
+      <c r="H65" t="s">
+        <v>808</v>
+      </c>
+      <c r="I65" t="s">
+        <v>809</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="s">
+        <v>833</v>
+      </c>
+      <c r="B66" t="s">
+        <v>850</v>
+      </c>
+      <c r="C66" t="n">
+        <v>17.15</v>
+      </c>
+      <c r="D66" t="s">
+        <v>857</v>
+      </c>
+      <c r="E66" t="s">
+        <v>835</v>
+      </c>
+      <c r="F66" t="n">
+        <v>198</v>
+      </c>
+      <c r="G66" t="s">
+        <v>834</v>
+      </c>
+      <c r="H66" t="s">
+        <v>835</v>
+      </c>
+      <c r="I66" t="s">
+        <v>836</v>
       </c>
     </row>
   </sheetData>

</xml_diff>